<commit_message>
Release ATS OneBSS 0.9.38
</commit_message>
<xml_diff>
--- a/Giao phiếu_demo2.xlsx
+++ b/Giao phiếu_demo2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranmanhcuong/Projects/ATS_OneBss/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{87BE9783-DEE4-3D48-94FC-8FCA5A79B12D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D8BAD60-B1E6-D74A-9296-39C2945054DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="105">
   <si>
     <t>Nhóm 1</t>
   </si>
@@ -376,7 +376,7 @@
       <family val="1"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -395,8 +395,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.79998168889431442"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="6">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -467,6 +473,19 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -522,19 +541,23 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -869,7 +892,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W31"/>
+  <dimension ref="A1:X31"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="17" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="8" customWidth="1"/>
@@ -890,39 +913,41 @@
     <col min="16" max="16" width="10.6640625" style="8" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="18.6640625" style="8" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="15.1640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="11" style="8" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="14.1640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="13.1640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="22" max="22" width="18.1640625" style="8" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="10.83203125" style="8" customWidth="1"/>
-    <col min="24" max="16384" width="10.83203125" style="8"/>
+    <col min="19" max="19" width="15.1640625" style="8" customWidth="1"/>
+    <col min="20" max="20" width="11" style="8" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="14.1640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="22" max="22" width="13.1640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="18.1640625" style="8" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="10.83203125" style="8" customWidth="1"/>
+    <col min="25" max="16384" width="10.83203125" style="8"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:23" x14ac:dyDescent="0.2">
-      <c r="E1" s="22" t="s">
+    <row r="1" spans="1:24" x14ac:dyDescent="0.2">
+      <c r="E1" s="24"/>
+      <c r="F1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="F1" s="23"/>
-      <c r="G1" s="23"/>
-      <c r="H1" s="23"/>
-      <c r="I1" s="23"/>
-      <c r="J1" s="23"/>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
-      <c r="M1" s="23"/>
-      <c r="N1" s="23"/>
-      <c r="O1" s="23"/>
-      <c r="P1" s="23"/>
-      <c r="Q1" s="23"/>
-      <c r="R1" s="24"/>
-      <c r="S1" s="19" t="s">
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+      <c r="M1" s="21"/>
+      <c r="N1" s="21"/>
+      <c r="O1" s="21"/>
+      <c r="P1" s="21"/>
+      <c r="Q1" s="21"/>
+      <c r="R1" s="21"/>
+      <c r="S1" s="23"/>
+      <c r="T1" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="T1" s="20"/>
-      <c r="U1" s="20"/>
-      <c r="V1" s="21"/>
-    </row>
-    <row r="2" spans="1:23" ht="35" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="U1" s="19"/>
+      <c r="V1" s="19"/>
+      <c r="W1" s="20"/>
+    </row>
+    <row r="2" spans="1:24" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
@@ -981,19 +1006,22 @@
         <v>21</v>
       </c>
       <c r="T2" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="U2" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="U2" s="3" t="s">
+      <c r="V2" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="V2" s="3" t="s">
+      <c r="W2" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="W2" s="9" t="s">
+      <c r="X2" s="9" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="3" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A3" s="9">
         <v>1</v>
       </c>
@@ -1025,12 +1053,13 @@
       <c r="S3" s="14">
         <v>0.5</v>
       </c>
-      <c r="T3" s="1"/>
+      <c r="T3" s="14"/>
       <c r="U3" s="1"/>
       <c r="V3" s="1"/>
-      <c r="W3" s="9"/>
-    </row>
-    <row r="4" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W3" s="1"/>
+      <c r="X3" s="9"/>
+    </row>
+    <row r="4" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A4" s="9">
         <v>2</v>
       </c>
@@ -1054,18 +1083,21 @@
       <c r="O4" s="1"/>
       <c r="P4" s="1"/>
       <c r="Q4" s="14">
-        <v>0.3</v>
-      </c>
-      <c r="R4" s="1"/>
+        <v>0.33</v>
+      </c>
+      <c r="R4" s="14">
+        <v>0.34</v>
+      </c>
       <c r="S4" s="14">
-        <v>0.7</v>
-      </c>
-      <c r="T4" s="1"/>
+        <v>0.33</v>
+      </c>
+      <c r="T4" s="14"/>
       <c r="U4" s="1"/>
       <c r="V4" s="1"/>
-      <c r="W4" s="9"/>
-    </row>
-    <row r="5" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W4" s="1"/>
+      <c r="X4" s="9"/>
+    </row>
+    <row r="5" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A5" s="9">
         <v>3</v>
       </c>
@@ -1096,9 +1128,10 @@
       <c r="T5" s="1"/>
       <c r="U5" s="1"/>
       <c r="V5" s="1"/>
-      <c r="W5" s="9"/>
-    </row>
-    <row r="6" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W5" s="1"/>
+      <c r="X5" s="9"/>
+    </row>
+    <row r="6" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A6" s="9">
         <v>4</v>
       </c>
@@ -1128,12 +1161,13 @@
       <c r="S6" s="14">
         <v>0.7</v>
       </c>
-      <c r="T6" s="1"/>
+      <c r="T6" s="14"/>
       <c r="U6" s="1"/>
       <c r="V6" s="1"/>
-      <c r="W6" s="9"/>
-    </row>
-    <row r="7" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W6" s="1"/>
+      <c r="X6" s="9"/>
+    </row>
+    <row r="7" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A7" s="9">
         <v>5</v>
       </c>
@@ -1174,11 +1208,12 @@
       <c r="T7" s="1"/>
       <c r="U7" s="1"/>
       <c r="V7" s="1"/>
-      <c r="W7" s="9" t="s">
+      <c r="W7" s="1"/>
+      <c r="X7" s="9" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="8" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A8" s="9">
         <v>6</v>
       </c>
@@ -1210,12 +1245,13 @@
       <c r="S8" s="14">
         <v>0.6</v>
       </c>
-      <c r="T8" s="1"/>
+      <c r="T8" s="14"/>
       <c r="U8" s="1"/>
       <c r="V8" s="1"/>
-      <c r="W8" s="9"/>
-    </row>
-    <row r="9" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W8" s="1"/>
+      <c r="X8" s="9"/>
+    </row>
+    <row r="9" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A9" s="9">
         <v>7</v>
       </c>
@@ -1247,12 +1283,13 @@
       <c r="S9" s="14">
         <v>0.6</v>
       </c>
-      <c r="T9" s="1"/>
+      <c r="T9" s="14"/>
       <c r="U9" s="1"/>
       <c r="V9" s="1"/>
-      <c r="W9" s="9"/>
-    </row>
-    <row r="10" spans="1:23" ht="108" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W9" s="1"/>
+      <c r="X9" s="9"/>
+    </row>
+    <row r="10" spans="1:24" ht="108" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="9">
         <v>8</v>
       </c>
@@ -1279,15 +1316,16 @@
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
       <c r="R10" s="1"/>
-      <c r="S10" s="14">
+      <c r="S10" s="1"/>
+      <c r="T10" s="14">
         <v>1</v>
       </c>
-      <c r="T10" s="14"/>
       <c r="U10" s="14"/>
       <c r="V10" s="14"/>
-      <c r="W10" s="9"/>
-    </row>
-    <row r="11" spans="1:23" ht="108" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W10" s="14"/>
+      <c r="X10" s="9"/>
+    </row>
+    <row r="11" spans="1:24" ht="108" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="9"/>
       <c r="B11" s="7" t="s">
         <v>104</v>
@@ -1312,19 +1350,20 @@
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
       <c r="R11" s="1"/>
-      <c r="S11" s="14"/>
-      <c r="T11" s="14">
+      <c r="S11" s="1"/>
+      <c r="T11" s="14"/>
+      <c r="U11" s="14">
         <v>0.34</v>
-      </c>
-      <c r="U11" s="14">
-        <v>0.33</v>
       </c>
       <c r="V11" s="14">
         <v>0.33</v>
       </c>
-      <c r="W11" s="9"/>
-    </row>
-    <row r="12" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W11" s="14">
+        <v>0.33</v>
+      </c>
+      <c r="X11" s="9"/>
+    </row>
+    <row r="12" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A12" s="9">
         <v>9</v>
       </c>
@@ -1357,9 +1396,10 @@
       <c r="T12" s="1"/>
       <c r="U12" s="1"/>
       <c r="V12" s="1"/>
-      <c r="W12" s="9"/>
-    </row>
-    <row r="13" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W12" s="1"/>
+      <c r="X12" s="9"/>
+    </row>
+    <row r="13" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A13" s="9">
         <v>10</v>
       </c>
@@ -1392,9 +1432,10 @@
       <c r="T13" s="1"/>
       <c r="U13" s="1"/>
       <c r="V13" s="1"/>
-      <c r="W13" s="9"/>
-    </row>
-    <row r="14" spans="1:23" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W13" s="1"/>
+      <c r="X13" s="9"/>
+    </row>
+    <row r="14" spans="1:24" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A14" s="9">
         <v>11</v>
       </c>
@@ -1437,11 +1478,12 @@
       <c r="T14" s="1"/>
       <c r="U14" s="1"/>
       <c r="V14" s="1"/>
-      <c r="W14" s="9" t="s">
+      <c r="W14" s="1"/>
+      <c r="X14" s="9" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:23" ht="54" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:24" ht="54" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="9">
         <v>12</v>
       </c>
@@ -1484,11 +1526,12 @@
       <c r="T15" s="1"/>
       <c r="U15" s="1"/>
       <c r="V15" s="1"/>
-      <c r="W15" s="9" t="s">
+      <c r="W15" s="1"/>
+      <c r="X15" s="9" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="16" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A16" s="9">
         <v>13</v>
       </c>
@@ -1525,11 +1568,12 @@
       <c r="T16" s="1"/>
       <c r="U16" s="1"/>
       <c r="V16" s="1"/>
-      <c r="W16" s="9" t="s">
+      <c r="W16" s="1"/>
+      <c r="X16" s="9" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="17" spans="1:23" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A17" s="9">
         <v>14</v>
       </c>
@@ -1560,9 +1604,10 @@
       <c r="T17" s="1"/>
       <c r="U17" s="1"/>
       <c r="V17" s="1"/>
-      <c r="W17" s="9"/>
-    </row>
-    <row r="18" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W17" s="1"/>
+      <c r="X17" s="9"/>
+    </row>
+    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A18" s="9">
         <v>15</v>
       </c>
@@ -1593,9 +1638,10 @@
       <c r="T18" s="1"/>
       <c r="U18" s="1"/>
       <c r="V18" s="1"/>
-      <c r="W18" s="9"/>
-    </row>
-    <row r="19" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W18" s="1"/>
+      <c r="X18" s="9"/>
+    </row>
+    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A19" s="9">
         <v>16</v>
       </c>
@@ -1628,9 +1674,10 @@
       <c r="T19" s="1"/>
       <c r="U19" s="1"/>
       <c r="V19" s="1"/>
-      <c r="W19" s="9"/>
-    </row>
-    <row r="20" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W19" s="1"/>
+      <c r="X19" s="9"/>
+    </row>
+    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A20" s="9">
         <v>17</v>
       </c>
@@ -1661,9 +1708,10 @@
       <c r="T20" s="1"/>
       <c r="U20" s="1"/>
       <c r="V20" s="1"/>
-      <c r="W20" s="9"/>
-    </row>
-    <row r="21" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W20" s="1"/>
+      <c r="X20" s="9"/>
+    </row>
+    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A21" s="9">
         <v>18</v>
       </c>
@@ -1696,9 +1744,10 @@
       <c r="T21" s="1"/>
       <c r="U21" s="1"/>
       <c r="V21" s="1"/>
-      <c r="W21" s="9"/>
-    </row>
-    <row r="22" spans="1:23" ht="72" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W21" s="1"/>
+      <c r="X21" s="9"/>
+    </row>
+    <row r="22" spans="1:24" ht="72" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A22" s="9">
         <v>19</v>
       </c>
@@ -1737,15 +1786,16 @@
       <c r="T22" s="1"/>
       <c r="U22" s="1"/>
       <c r="V22" s="1"/>
-      <c r="W22" s="9" t="s">
+      <c r="W22" s="1"/>
+      <c r="X22" s="9" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="23" spans="1:23" ht="18" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:24" ht="18" x14ac:dyDescent="0.2">
       <c r="A23" s="9">
         <v>20</v>
       </c>
-      <c r="B23" s="18" t="s">
+      <c r="B23" s="7" t="s">
         <v>98</v>
       </c>
       <c r="C23" s="10">
@@ -1776,13 +1826,14 @@
       <c r="T23" s="1"/>
       <c r="U23" s="1"/>
       <c r="V23" s="1"/>
-      <c r="W23" s="9"/>
-    </row>
-    <row r="24" spans="1:23" ht="18" x14ac:dyDescent="0.2">
+      <c r="W23" s="1"/>
+      <c r="X23" s="9"/>
+    </row>
+    <row r="24" spans="1:24" ht="18" x14ac:dyDescent="0.2">
       <c r="A24" s="9">
         <v>21</v>
       </c>
-      <c r="B24" s="18" t="s">
+      <c r="B24" s="7" t="s">
         <v>99</v>
       </c>
       <c r="C24" s="10">
@@ -1811,9 +1862,10 @@
       <c r="T24" s="1"/>
       <c r="U24" s="1"/>
       <c r="V24" s="1"/>
-      <c r="W24" s="9"/>
-    </row>
-    <row r="25" spans="1:23" ht="90" x14ac:dyDescent="0.2">
+      <c r="W24" s="1"/>
+      <c r="X24" s="9"/>
+    </row>
+    <row r="25" spans="1:24" ht="90" x14ac:dyDescent="0.2">
       <c r="A25" s="9">
         <v>22</v>
       </c>
@@ -1848,9 +1900,10 @@
       <c r="T25" s="1"/>
       <c r="U25" s="1"/>
       <c r="V25" s="1"/>
-      <c r="W25" s="9"/>
-    </row>
-    <row r="26" spans="1:23" ht="36" x14ac:dyDescent="0.2">
+      <c r="W25" s="1"/>
+      <c r="X25" s="9"/>
+    </row>
+    <row r="26" spans="1:24" ht="36" x14ac:dyDescent="0.2">
       <c r="A26" s="9">
         <v>23</v>
       </c>
@@ -1883,9 +1936,10 @@
       <c r="T26" s="1"/>
       <c r="U26" s="1"/>
       <c r="V26" s="1"/>
-      <c r="W26" s="9"/>
-    </row>
-    <row r="27" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W26" s="1"/>
+      <c r="X26" s="9"/>
+    </row>
+    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A27" s="9">
         <v>24</v>
       </c>
@@ -1916,9 +1970,10 @@
       <c r="T27" s="1"/>
       <c r="U27" s="1"/>
       <c r="V27" s="1"/>
-      <c r="W27" s="9"/>
-    </row>
-    <row r="28" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W27" s="1"/>
+      <c r="X27" s="9"/>
+    </row>
+    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A28" s="9">
         <v>25</v>
       </c>
@@ -1943,9 +1998,7 @@
       <c r="P28" s="1"/>
       <c r="Q28" s="1"/>
       <c r="R28" s="1"/>
-      <c r="S28" s="14">
-        <v>0.25</v>
-      </c>
+      <c r="S28" s="1"/>
       <c r="T28" s="14">
         <v>0.25</v>
       </c>
@@ -1955,9 +2008,12 @@
       <c r="V28" s="14">
         <v>0.25</v>
       </c>
-      <c r="W28" s="9"/>
-    </row>
-    <row r="29" spans="1:23" x14ac:dyDescent="0.2">
+      <c r="W28" s="14">
+        <v>0.25</v>
+      </c>
+      <c r="X28" s="9"/>
+    </row>
+    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A29" s="9">
         <v>26</v>
       </c>
@@ -1984,13 +2040,14 @@
       <c r="R29" s="14">
         <v>1</v>
       </c>
-      <c r="S29" s="1"/>
+      <c r="S29" s="14"/>
       <c r="T29" s="1"/>
       <c r="U29" s="1"/>
       <c r="V29" s="1"/>
-      <c r="W29" s="9"/>
-    </row>
-    <row r="30" spans="1:23" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="W29" s="1"/>
+      <c r="X29" s="9"/>
+    </row>
+    <row r="30" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A30" s="9">
         <v>27</v>
       </c>
@@ -2022,8 +2079,9 @@
       <c r="U30" s="9"/>
       <c r="V30" s="9"/>
       <c r="W30" s="9"/>
-    </row>
-    <row r="31" spans="1:23" ht="36" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="X30" s="9"/>
+    </row>
+    <row r="31" spans="1:24" ht="36" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="9">
         <v>28</v>
       </c>
@@ -2055,11 +2113,12 @@
       <c r="U31" s="9"/>
       <c r="V31" s="9"/>
       <c r="W31" s="9"/>
+      <c r="X31" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="S1:V1"/>
-    <mergeCell ref="E1:R1"/>
+    <mergeCell ref="T1:W1"/>
+    <mergeCell ref="F1:S1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>

<commit_message>
Restore North release from 0.9.64 with latest calendar and rules
</commit_message>
<xml_diff>
--- a/Giao phiếu_demo2.xlsx
+++ b/Giao phiếu_demo2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="11020"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tranmanhcuong/Projects/ATS_OneBss/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D8BAD60-B1E6-D74A-9296-39C2945054DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4F05349-781A-8F44-AFFA-9521B834C9A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="51200" windowHeight="21000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="51200" yWindow="10300" windowWidth="30240" windowHeight="18980" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Quy tắc giao phiếu" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="271" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="300" uniqueCount="108">
   <si>
     <t>Nhóm 1</t>
   </si>
@@ -321,9 +321,6 @@
     <t>Kiểu lắp đặt: Gia hạn và thay đổi gói cước CNTT/GTGT, Gia hạn dịch vụ CNTT/GTGT, Chấm dứt sử dụng, Thanh lý dịch vụ CNTT/GTGT - qua Vip, Thanh lý DV CNTT</t>
   </si>
   <si>
-    <t>Kiểu lắp đặt: Thay đổi thông tin DV CNTT/GTGT</t>
-  </si>
-  <si>
     <t>Quy tắc group</t>
   </si>
   <si>
@@ -349,6 +346,18 @@
   </si>
   <si>
     <t>Voice Brandname XL</t>
+  </si>
+  <si>
+    <t>Megawan quang GE</t>
+  </si>
+  <si>
+    <t>Leasedline 100GE</t>
+  </si>
+  <si>
+    <t>Megawan ADSL</t>
+  </si>
+  <si>
+    <t>Kiểu lắp đặt: Thay đổi thông tin DV CNTT/GTGT, Yêu cầu Vip hỗ trợ: TTKD-Vip-TTKD - Không thay đổi TTKH</t>
   </si>
 </sst>
 </file>
@@ -541,22 +550,22 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -923,29 +932,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:24" x14ac:dyDescent="0.2">
-      <c r="E1" s="24"/>
+      <c r="E1" s="18"/>
       <c r="F1" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="G1" s="21"/>
-      <c r="H1" s="21"/>
-      <c r="I1" s="21"/>
-      <c r="J1" s="21"/>
-      <c r="K1" s="21"/>
-      <c r="L1" s="21"/>
-      <c r="M1" s="21"/>
-      <c r="N1" s="21"/>
-      <c r="O1" s="21"/>
-      <c r="P1" s="21"/>
-      <c r="Q1" s="21"/>
-      <c r="R1" s="21"/>
-      <c r="S1" s="23"/>
-      <c r="T1" s="18" t="s">
+      <c r="G1" s="23"/>
+      <c r="H1" s="23"/>
+      <c r="I1" s="23"/>
+      <c r="J1" s="23"/>
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+      <c r="M1" s="23"/>
+      <c r="N1" s="23"/>
+      <c r="O1" s="23"/>
+      <c r="P1" s="23"/>
+      <c r="Q1" s="23"/>
+      <c r="R1" s="23"/>
+      <c r="S1" s="24"/>
+      <c r="T1" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="U1" s="19"/>
-      <c r="V1" s="19"/>
-      <c r="W1" s="20"/>
+      <c r="U1" s="20"/>
+      <c r="V1" s="20"/>
+      <c r="W1" s="21"/>
     </row>
     <row r="2" spans="1:24" ht="35" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
@@ -1294,13 +1303,13 @@
         <v>8</v>
       </c>
       <c r="B10" s="7" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C10" s="10">
         <v>20</v>
       </c>
       <c r="D10" s="10" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E10" s="10"/>
       <c r="F10" s="1"/>
@@ -1328,13 +1337,13 @@
     <row r="11" spans="1:24" ht="108" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="9"/>
       <c r="B11" s="7" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C11" s="10">
         <v>20</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="E11" s="10"/>
       <c r="F11" s="1"/>
@@ -1450,7 +1459,7 @@
       </c>
       <c r="E14" s="10"/>
       <c r="F14" s="14">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="G14" s="14">
         <v>0.1</v>
@@ -1459,18 +1468,26 @@
         <v>0.1</v>
       </c>
       <c r="I14" s="1"/>
-      <c r="J14" s="1"/>
+      <c r="J14" s="14">
+        <v>0.1</v>
+      </c>
       <c r="K14" s="14">
         <v>0.1</v>
       </c>
-      <c r="L14" s="1"/>
-      <c r="M14" s="1"/>
-      <c r="N14" s="1"/>
+      <c r="L14" s="14">
+        <v>0.1</v>
+      </c>
+      <c r="M14" s="14">
+        <v>0.1</v>
+      </c>
+      <c r="N14" s="14">
+        <v>0.1</v>
+      </c>
       <c r="O14" s="14">
         <v>0.1</v>
       </c>
       <c r="P14" s="14">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="Q14" s="1"/>
       <c r="R14" s="1"/>
@@ -1498,7 +1515,7 @@
       </c>
       <c r="E15" s="10"/>
       <c r="F15" s="14">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="G15" s="14">
         <v>0.1</v>
@@ -1507,18 +1524,26 @@
         <v>0.1</v>
       </c>
       <c r="I15" s="1"/>
-      <c r="J15" s="1"/>
+      <c r="J15" s="14">
+        <v>0.1</v>
+      </c>
       <c r="K15" s="14">
         <v>0.1</v>
       </c>
-      <c r="L15" s="1"/>
-      <c r="M15" s="1"/>
-      <c r="N15" s="1"/>
+      <c r="L15" s="14">
+        <v>0.1</v>
+      </c>
+      <c r="M15" s="14">
+        <v>0.1</v>
+      </c>
+      <c r="N15" s="14">
+        <v>0.1</v>
+      </c>
       <c r="O15" s="14">
         <v>0.1</v>
       </c>
       <c r="P15" s="14">
-        <v>0.3</v>
+        <v>0.1</v>
       </c>
       <c r="Q15" s="1"/>
       <c r="R15" s="1"/>
@@ -1796,7 +1821,7 @@
         <v>20</v>
       </c>
       <c r="B23" s="7" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C23" s="10">
         <v>29</v>
@@ -1834,7 +1859,7 @@
         <v>21</v>
       </c>
       <c r="B24" s="7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C24" s="10">
         <v>29</v>
@@ -1870,7 +1895,7 @@
         <v>22</v>
       </c>
       <c r="B25" s="7" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C25" s="10">
         <v>14</v>
@@ -1903,18 +1928,18 @@
       <c r="W25" s="1"/>
       <c r="X25" s="9"/>
     </row>
-    <row r="26" spans="1:24" ht="36" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:24" ht="54" x14ac:dyDescent="0.2">
       <c r="A26" s="9">
         <v>23</v>
       </c>
       <c r="B26" s="7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C26" s="10">
         <v>14</v>
       </c>
       <c r="D26" s="11" t="s">
-        <v>95</v>
+        <v>107</v>
       </c>
       <c r="E26" s="11"/>
       <c r="F26" s="1"/>
@@ -2127,7 +2152,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4DE81EBB-08AC-CB41-ACC3-3E8E86C36875}">
-  <dimension ref="A1:F61"/>
+  <dimension ref="A1:F66"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
@@ -2152,7 +2177,7 @@
         <v>5</v>
       </c>
       <c r="E1" s="15" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F1" s="15" t="s">
         <v>89</v>
@@ -2386,7 +2411,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A14" s="9">
         <v>13</v>
       </c>
@@ -2399,12 +2424,14 @@
       <c r="D14" s="10">
         <v>17</v>
       </c>
-      <c r="E14" s="10"/>
+      <c r="E14" s="11" t="s">
+        <v>43</v>
+      </c>
       <c r="F14" s="13" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" ht="72" x14ac:dyDescent="0.2">
       <c r="A15" s="9">
         <v>14</v>
       </c>
@@ -2417,53 +2444,59 @@
       <c r="D15" s="10">
         <v>27</v>
       </c>
-      <c r="E15" s="10"/>
+      <c r="E15" s="6" t="s">
+        <v>48</v>
+      </c>
       <c r="F15" s="13" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A16" s="9">
         <v>15</v>
       </c>
       <c r="B16" s="9" t="s">
-        <v>74</v>
+        <v>104</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D16" s="10">
         <v>17</v>
       </c>
-      <c r="E16" s="10"/>
+      <c r="E16" s="11" t="s">
+        <v>43</v>
+      </c>
       <c r="F16" s="13" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" ht="72" x14ac:dyDescent="0.2">
       <c r="A17" s="9">
         <v>16</v>
       </c>
       <c r="B17" s="9" t="s">
-        <v>74</v>
-      </c>
-      <c r="C17" s="7" t="s">
-        <v>49</v>
+        <v>104</v>
+      </c>
+      <c r="C17" s="9" t="s">
+        <v>47</v>
       </c>
       <c r="D17" s="10">
         <v>27</v>
       </c>
-      <c r="E17" s="10"/>
+      <c r="E17" s="6" t="s">
+        <v>48</v>
+      </c>
       <c r="F17" s="13" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A18" s="9">
         <v>17</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>45</v>
@@ -2471,17 +2504,19 @@
       <c r="D18" s="10">
         <v>17</v>
       </c>
-      <c r="E18" s="10"/>
+      <c r="E18" s="11" t="s">
+        <v>43</v>
+      </c>
       <c r="F18" s="13" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" ht="72" x14ac:dyDescent="0.2">
       <c r="A19" s="9">
         <v>18</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C19" s="7" t="s">
         <v>49</v>
@@ -2489,17 +2524,19 @@
       <c r="D19" s="10">
         <v>27</v>
       </c>
-      <c r="E19" s="10"/>
+      <c r="E19" s="6" t="s">
+        <v>48</v>
+      </c>
       <c r="F19" s="13" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A20" s="9">
         <v>19</v>
       </c>
       <c r="B20" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C20" s="7" t="s">
         <v>45</v>
@@ -2507,17 +2544,19 @@
       <c r="D20" s="10">
         <v>17</v>
       </c>
-      <c r="E20" s="10"/>
+      <c r="E20" s="11" t="s">
+        <v>43</v>
+      </c>
       <c r="F20" s="13" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" ht="72" x14ac:dyDescent="0.2">
       <c r="A21" s="9">
         <v>20</v>
       </c>
       <c r="B21" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C21" s="7" t="s">
         <v>49</v>
@@ -2525,133 +2564,147 @@
       <c r="D21" s="10">
         <v>27</v>
       </c>
-      <c r="E21" s="10"/>
+      <c r="E21" s="6" t="s">
+        <v>48</v>
+      </c>
       <c r="F21" s="13" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="22" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A22" s="9">
         <v>21</v>
       </c>
       <c r="B22" s="9" t="s">
-        <v>83</v>
+        <v>76</v>
       </c>
       <c r="C22" s="7" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="D22" s="10">
         <v>17</v>
       </c>
-      <c r="E22" s="10"/>
+      <c r="E22" s="11" t="s">
+        <v>43</v>
+      </c>
       <c r="F22" s="13" t="s">
         <v>90</v>
       </c>
     </row>
-    <row r="23" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" ht="72" x14ac:dyDescent="0.2">
       <c r="A23" s="9">
         <v>22</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>83</v>
-      </c>
-      <c r="C23" s="9" t="s">
-        <v>47</v>
+        <v>76</v>
+      </c>
+      <c r="C23" s="7" t="s">
+        <v>49</v>
       </c>
       <c r="D23" s="10">
         <v>27</v>
       </c>
-      <c r="E23" s="10"/>
+      <c r="E23" s="6" t="s">
+        <v>48</v>
+      </c>
       <c r="F23" s="13" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="24" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A24" s="9">
         <v>23</v>
       </c>
-      <c r="B24" s="7" t="s">
-        <v>59</v>
+      <c r="B24" s="9" t="s">
+        <v>83</v>
       </c>
       <c r="C24" s="7" t="s">
-        <v>60</v>
+        <v>42</v>
       </c>
       <c r="D24" s="10">
-        <v>42</v>
-      </c>
-      <c r="E24" s="10"/>
-      <c r="F24" s="7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+        <v>17</v>
+      </c>
+      <c r="E24" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" ht="72" x14ac:dyDescent="0.2">
       <c r="A25" s="9">
         <v>24</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C25" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="D25" s="9">
-        <v>42</v>
-      </c>
-      <c r="E25" s="9"/>
-      <c r="F25" s="7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+        <v>47</v>
+      </c>
+      <c r="D25" s="10">
+        <v>27</v>
+      </c>
+      <c r="E25" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A26" s="9">
         <v>25</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>78</v>
-      </c>
-      <c r="C26" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="D26" s="9">
+        <v>106</v>
+      </c>
+      <c r="C26" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="E26" s="9"/>
-      <c r="F26" s="7" t="s">
-        <v>60</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="D26" s="10">
+        <v>17</v>
+      </c>
+      <c r="E26" s="11" t="s">
+        <v>43</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" ht="72" x14ac:dyDescent="0.2">
       <c r="A27" s="9">
         <v>26</v>
       </c>
       <c r="B27" s="9" t="s">
-        <v>79</v>
+        <v>106</v>
       </c>
       <c r="C27" s="9" t="s">
-        <v>60</v>
-      </c>
-      <c r="D27" s="9">
-        <v>42</v>
-      </c>
-      <c r="E27" s="9"/>
-      <c r="F27" s="7" t="s">
-        <v>60</v>
+        <v>47</v>
+      </c>
+      <c r="D27" s="10">
+        <v>27</v>
+      </c>
+      <c r="E27" s="6" t="s">
+        <v>48</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>91</v>
       </c>
     </row>
     <row r="28" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A28" s="9">
         <v>27</v>
       </c>
-      <c r="B28" s="9" t="s">
-        <v>82</v>
-      </c>
-      <c r="C28" s="9" t="s">
+      <c r="B28" s="7" t="s">
+        <v>59</v>
+      </c>
+      <c r="C28" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="D28" s="9">
+      <c r="D28" s="10">
         <v>42</v>
       </c>
-      <c r="E28" s="9"/>
+      <c r="E28" s="10"/>
       <c r="F28" s="7" t="s">
         <v>60</v>
       </c>
@@ -2660,340 +2713,340 @@
       <c r="A29" s="9">
         <v>28</v>
       </c>
-      <c r="B29" s="7">
-        <v>1800</v>
-      </c>
-      <c r="C29" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D29" s="10">
-        <v>17</v>
-      </c>
-      <c r="E29" s="10"/>
+      <c r="B29" s="9" t="s">
+        <v>77</v>
+      </c>
+      <c r="C29" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D29" s="9">
+        <v>42</v>
+      </c>
+      <c r="E29" s="9"/>
       <c r="F29" s="7" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
     </row>
     <row r="30" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A30" s="9">
         <v>29</v>
       </c>
-      <c r="B30" s="7">
-        <v>1900</v>
-      </c>
-      <c r="C30" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D30" s="10">
-        <v>17</v>
-      </c>
-      <c r="E30" s="10"/>
+      <c r="B30" s="9" t="s">
+        <v>78</v>
+      </c>
+      <c r="C30" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D30" s="9">
+        <v>42</v>
+      </c>
+      <c r="E30" s="9"/>
       <c r="F30" s="7" t="s">
-        <v>37</v>
+        <v>60</v>
       </c>
     </row>
     <row r="31" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A31" s="9">
         <v>30</v>
       </c>
-      <c r="B31" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="C31" s="7" t="s">
-        <v>52</v>
-      </c>
-      <c r="D31" s="10">
-        <v>27</v>
-      </c>
-      <c r="E31" s="10"/>
+      <c r="B31" s="9" t="s">
+        <v>79</v>
+      </c>
+      <c r="C31" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D31" s="9">
+        <v>42</v>
+      </c>
+      <c r="E31" s="9"/>
       <c r="F31" s="7" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="32" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A32" s="9">
         <v>31</v>
       </c>
-      <c r="B32" s="7" t="s">
-        <v>53</v>
-      </c>
-      <c r="C32" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D32" s="10">
-        <v>27</v>
-      </c>
-      <c r="E32" s="10"/>
+      <c r="B32" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C32" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D32" s="9">
+        <v>42</v>
+      </c>
+      <c r="E32" s="9"/>
       <c r="F32" s="7" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
     </row>
     <row r="33" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A33" s="9">
         <v>32</v>
       </c>
-      <c r="B33" s="7" t="s">
-        <v>55</v>
-      </c>
-      <c r="C33" s="7" t="s">
-        <v>54</v>
-      </c>
-      <c r="D33" s="10">
-        <v>27</v>
-      </c>
-      <c r="E33" s="10"/>
+      <c r="B33" s="9" t="s">
+        <v>105</v>
+      </c>
+      <c r="C33" s="9" t="s">
+        <v>60</v>
+      </c>
+      <c r="D33" s="9">
+        <v>42</v>
+      </c>
+      <c r="E33" s="9"/>
       <c r="F33" s="7" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" ht="108" x14ac:dyDescent="0.2">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A34" s="9">
         <v>33</v>
       </c>
-      <c r="B34" s="7" t="s">
-        <v>62</v>
+      <c r="B34" s="7">
+        <v>1800</v>
       </c>
       <c r="C34" s="7" t="s">
-        <v>63</v>
+        <v>37</v>
       </c>
       <c r="D34" s="10">
-        <v>14</v>
-      </c>
-      <c r="E34" s="11" t="s">
-        <v>94</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="E34" s="10"/>
       <c r="F34" s="7" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="108" x14ac:dyDescent="0.2">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A35" s="9">
         <v>34</v>
       </c>
-      <c r="B35" s="7" t="s">
-        <v>64</v>
+      <c r="B35" s="7">
+        <v>1900</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>65</v>
+        <v>37</v>
       </c>
       <c r="D35" s="10">
-        <v>14</v>
-      </c>
-      <c r="E35" s="11" t="s">
-        <v>94</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="E35" s="10"/>
       <c r="F35" s="7" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" ht="18" x14ac:dyDescent="0.2">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A36" s="9">
         <v>35</v>
       </c>
       <c r="B36" s="7" t="s">
-        <v>62</v>
+        <v>52</v>
       </c>
       <c r="C36" s="7" t="s">
-        <v>66</v>
+        <v>52</v>
       </c>
       <c r="D36" s="10">
-        <v>29</v>
-      </c>
-      <c r="E36" s="11" t="s">
-        <v>93</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="E36" s="10"/>
       <c r="F36" s="7" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" ht="18" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A37" s="9">
         <v>36</v>
       </c>
       <c r="B37" s="7" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="C37" s="7" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="D37" s="10">
-        <v>29</v>
-      </c>
-      <c r="E37" s="11" t="s">
-        <v>93</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="E37" s="10"/>
       <c r="F37" s="7" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" ht="36" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A38" s="9">
         <v>37</v>
       </c>
       <c r="B38" s="7" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C38" s="7" t="s">
-        <v>66</v>
+        <v>54</v>
       </c>
       <c r="D38" s="10">
-        <v>29</v>
-      </c>
-      <c r="E38" s="11" t="s">
-        <v>92</v>
-      </c>
+        <v>27</v>
+      </c>
+      <c r="E38" s="10"/>
       <c r="F38" s="7" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" ht="36" x14ac:dyDescent="0.2">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" ht="108" x14ac:dyDescent="0.2">
       <c r="A39" s="9">
         <v>38</v>
       </c>
       <c r="B39" s="7" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C39" s="7" t="s">
-        <v>67</v>
+        <v>63</v>
       </c>
       <c r="D39" s="10">
-        <v>29</v>
+        <v>14</v>
       </c>
       <c r="E39" s="11" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F39" s="7" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" ht="36" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" ht="108" x14ac:dyDescent="0.2">
       <c r="A40" s="9">
         <v>39</v>
       </c>
       <c r="B40" s="7" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C40" s="7" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D40" s="10">
         <v>14</v>
       </c>
       <c r="E40" s="11" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F40" s="7" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" ht="36" x14ac:dyDescent="0.2">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A41" s="9">
         <v>40</v>
       </c>
       <c r="B41" s="7" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="C41" s="7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="D41" s="10">
-        <v>14</v>
+        <v>29</v>
       </c>
       <c r="E41" s="11" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="F41" s="7" t="s">
-        <v>100</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" ht="18" x14ac:dyDescent="0.2">
       <c r="A42" s="9">
         <v>41</v>
       </c>
       <c r="B42" s="7" t="s">
+        <v>64</v>
+      </c>
+      <c r="C42" s="7" t="s">
+        <v>67</v>
+      </c>
+      <c r="D42" s="10">
         <v>29</v>
       </c>
-      <c r="C42" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="D42" s="10">
-        <v>10</v>
-      </c>
-      <c r="E42" s="10"/>
+      <c r="E42" s="11" t="s">
+        <v>93</v>
+      </c>
       <c r="F42" s="7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" ht="36" x14ac:dyDescent="0.2">
       <c r="A43" s="9">
         <v>42</v>
       </c>
       <c r="B43" s="7" t="s">
-        <v>31</v>
+        <v>62</v>
       </c>
       <c r="C43" s="7" t="s">
-        <v>30</v>
+        <v>66</v>
       </c>
       <c r="D43" s="10">
-        <v>10</v>
-      </c>
-      <c r="E43" s="10"/>
+        <v>29</v>
+      </c>
+      <c r="E43" s="11" t="s">
+        <v>92</v>
+      </c>
       <c r="F43" s="7" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" ht="36" x14ac:dyDescent="0.2">
       <c r="A44" s="9">
         <v>43</v>
       </c>
       <c r="B44" s="7" t="s">
-        <v>68</v>
+        <v>64</v>
       </c>
       <c r="C44" s="7" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D44" s="10">
-        <v>17</v>
-      </c>
-      <c r="E44" s="10"/>
+        <v>29</v>
+      </c>
+      <c r="E44" s="11" t="s">
+        <v>92</v>
+      </c>
       <c r="F44" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" ht="72" x14ac:dyDescent="0.2">
       <c r="A45" s="9">
         <v>44</v>
       </c>
       <c r="B45" s="7" t="s">
-        <v>86</v>
+        <v>62</v>
       </c>
       <c r="C45" s="7" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="D45" s="10">
-        <v>17</v>
-      </c>
-      <c r="E45" s="10"/>
+        <v>14</v>
+      </c>
+      <c r="E45" s="11" t="s">
+        <v>107</v>
+      </c>
       <c r="F45" s="7" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" ht="72" x14ac:dyDescent="0.2">
       <c r="A46" s="9">
         <v>45</v>
       </c>
       <c r="B46" s="7" t="s">
-        <v>25</v>
+        <v>64</v>
       </c>
       <c r="C46" s="7" t="s">
-        <v>25</v>
+        <v>65</v>
       </c>
       <c r="D46" s="10">
-        <v>10</v>
-      </c>
-      <c r="E46" s="10"/>
+        <v>14</v>
+      </c>
+      <c r="E46" s="11" t="s">
+        <v>107</v>
+      </c>
       <c r="F46" s="7" t="s">
-        <v>25</v>
+        <v>99</v>
       </c>
     </row>
     <row r="47" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -3001,17 +3054,17 @@
         <v>46</v>
       </c>
       <c r="B47" s="7" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C47" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D47" s="10">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E47" s="10"/>
       <c r="F47" s="7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="48" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -3019,17 +3072,17 @@
         <v>47</v>
       </c>
       <c r="B48" s="7" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="C48" s="7" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D48" s="10">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E48" s="10"/>
       <c r="F48" s="7" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
     </row>
     <row r="49" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -3037,19 +3090,17 @@
         <v>48</v>
       </c>
       <c r="B49" s="7" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="C49" s="7" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="D49" s="10">
-        <v>20</v>
-      </c>
-      <c r="E49" s="10" t="s">
-        <v>101</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="E49" s="10"/>
       <c r="F49" s="7" t="s">
-        <v>103</v>
+        <v>68</v>
       </c>
     </row>
     <row r="50" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -3057,19 +3108,17 @@
         <v>49</v>
       </c>
       <c r="B50" s="7" t="s">
-        <v>38</v>
+        <v>86</v>
       </c>
       <c r="C50" s="7" t="s">
-        <v>38</v>
+        <v>68</v>
       </c>
       <c r="D50" s="10">
-        <v>20</v>
-      </c>
-      <c r="E50" s="10" t="s">
-        <v>102</v>
-      </c>
+        <v>17</v>
+      </c>
+      <c r="E50" s="10"/>
       <c r="F50" s="7" t="s">
-        <v>104</v>
+        <v>68</v>
       </c>
     </row>
     <row r="51" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -3077,17 +3126,17 @@
         <v>50</v>
       </c>
       <c r="B51" s="7" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="C51" s="7" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
       <c r="D51" s="10">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="E51" s="10"/>
       <c r="F51" s="7" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
     </row>
     <row r="52" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -3095,17 +3144,17 @@
         <v>51</v>
       </c>
       <c r="B52" s="7" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="C52" s="7" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="D52" s="10">
         <v>17</v>
       </c>
       <c r="E52" s="10"/>
       <c r="F52" s="7" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
     </row>
     <row r="53" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -3113,17 +3162,17 @@
         <v>52</v>
       </c>
       <c r="B53" s="7" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="C53" s="7" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
       <c r="D53" s="10">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E53" s="10"/>
       <c r="F53" s="7" t="s">
-        <v>46</v>
+        <v>36</v>
       </c>
     </row>
     <row r="54" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -3131,17 +3180,19 @@
         <v>53</v>
       </c>
       <c r="B54" s="7" t="s">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="C54" s="7" t="s">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="D54" s="10">
-        <v>27</v>
-      </c>
-      <c r="E54" s="10"/>
+        <v>20</v>
+      </c>
+      <c r="E54" s="10" t="s">
+        <v>100</v>
+      </c>
       <c r="F54" s="7" t="s">
-        <v>51</v>
+        <v>102</v>
       </c>
     </row>
     <row r="55" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -3149,17 +3200,19 @@
         <v>54</v>
       </c>
       <c r="B55" s="7" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="C55" s="7" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="D55" s="10">
-        <v>27</v>
-      </c>
-      <c r="E55" s="10"/>
+        <v>20</v>
+      </c>
+      <c r="E55" s="10" t="s">
+        <v>101</v>
+      </c>
       <c r="F55" s="7" t="s">
-        <v>56</v>
+        <v>103</v>
       </c>
     </row>
     <row r="56" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -3167,17 +3220,17 @@
         <v>55</v>
       </c>
       <c r="B56" s="7" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="C56" s="7" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
       <c r="D56" s="10">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E56" s="10"/>
       <c r="F56" s="7" t="s">
-        <v>57</v>
+        <v>39</v>
       </c>
     </row>
     <row r="57" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -3185,17 +3238,17 @@
         <v>56</v>
       </c>
       <c r="B57" s="7" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="C57" s="7" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="D57" s="10">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E57" s="10"/>
       <c r="F57" s="7" t="s">
-        <v>58</v>
+        <v>40</v>
       </c>
     </row>
     <row r="58" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -3203,17 +3256,17 @@
         <v>57</v>
       </c>
       <c r="B58" s="7" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="C58" s="7" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
       <c r="D58" s="10">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="E58" s="10"/>
       <c r="F58" s="7" t="s">
-        <v>69</v>
+        <v>46</v>
       </c>
     </row>
     <row r="59" spans="1:6" ht="17" x14ac:dyDescent="0.2">
@@ -3221,48 +3274,138 @@
         <v>58</v>
       </c>
       <c r="B59" s="7" t="s">
-        <v>70</v>
+        <v>50</v>
       </c>
       <c r="C59" s="7" t="s">
-        <v>71</v>
+        <v>51</v>
       </c>
       <c r="D59" s="10">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="E59" s="10"/>
       <c r="F59" s="7" t="s">
-        <v>71</v>
+        <v>51</v>
       </c>
     </row>
     <row r="60" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A60" s="9">
         <v>59</v>
       </c>
-      <c r="B60" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="C60" s="9" t="s">
-        <v>80</v>
-      </c>
-      <c r="D60" s="9"/>
-      <c r="E60" s="9"/>
-      <c r="F60" s="9" t="s">
-        <v>80</v>
+      <c r="B60" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="C60" s="7" t="s">
+        <v>56</v>
+      </c>
+      <c r="D60" s="10">
+        <v>27</v>
+      </c>
+      <c r="E60" s="10"/>
+      <c r="F60" s="7" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="61" spans="1:6" ht="17" x14ac:dyDescent="0.2">
       <c r="A61" s="9">
         <v>60</v>
       </c>
-      <c r="B61" s="9" t="s">
+      <c r="B61" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C61" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="D61" s="10">
+        <v>27</v>
+      </c>
+      <c r="E61" s="10"/>
+      <c r="F61" s="7" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A62" s="9">
+        <v>61</v>
+      </c>
+      <c r="B62" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="C62" s="7" t="s">
+        <v>58</v>
+      </c>
+      <c r="D62" s="10">
+        <v>27</v>
+      </c>
+      <c r="E62" s="10"/>
+      <c r="F62" s="7" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A63" s="9">
+        <v>62</v>
+      </c>
+      <c r="B63" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="C63" s="7" t="s">
+        <v>69</v>
+      </c>
+      <c r="D63" s="10">
+        <v>25</v>
+      </c>
+      <c r="E63" s="10"/>
+      <c r="F63" s="7" t="s">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A64" s="9">
+        <v>63</v>
+      </c>
+      <c r="B64" s="7" t="s">
+        <v>70</v>
+      </c>
+      <c r="C64" s="7" t="s">
+        <v>71</v>
+      </c>
+      <c r="D64" s="10">
+        <v>14</v>
+      </c>
+      <c r="E64" s="10"/>
+      <c r="F64" s="7" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A65" s="9">
+        <v>64</v>
+      </c>
+      <c r="B65" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="C65" s="9" t="s">
+        <v>80</v>
+      </c>
+      <c r="D65" s="9"/>
+      <c r="E65" s="9"/>
+      <c r="F65" s="9" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" ht="17" x14ac:dyDescent="0.2">
+      <c r="A66" s="9">
+        <v>65</v>
+      </c>
+      <c r="B66" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="C61" s="9" t="s">
+      <c r="C66" s="9" t="s">
         <v>84</v>
       </c>
-      <c r="D61" s="9"/>
-      <c r="E61" s="9"/>
-      <c r="F61" s="9" t="s">
+      <c r="D66" s="9"/>
+      <c r="E66" s="9"/>
+      <c r="F66" s="9" t="s">
         <v>84</v>
       </c>
     </row>

</xml_diff>